<commit_message>
staged parser codes and note that duplicates produced in odakyu table when running retrieve_by_neighbours
</commit_message>
<xml_diff>
--- a/result/odakyu-stops-final-2024-05-06.xlsx
+++ b/result/odakyu-stops-final-2024-05-06.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mario/github/google-poi-japan/result/odakyu-stops-updated-2024-05-06 14:13:"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mario/github/google-poi-japan/result/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58624638-BEA9-8D40-8037-4F88EF63ADA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97BEB51B-CAE3-FA48-8AA0-10EBC28DE99B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="462">
   <si>
     <t>formatted_address</t>
   </si>
@@ -76,15 +76,6 @@
     <t>Tokyo, Japan</t>
   </si>
   <si>
-    <t>Shinjuku City, Tokyo, Japan</t>
-  </si>
-  <si>
-    <t>{'location': {'lat': 35.6905539, 'lng': 139.6995499}, 'viewport': {'northeast': {'lat': 35.69190372989272, 'lng': 139.7008997298927}, 'southwest': {'lat': 35.68920407010727, 'lng': 139.6982000701072}}}</t>
-  </si>
-  <si>
-    <t>ChIJu9ljKNeMGGARcFUr-NmJhAk</t>
-  </si>
-  <si>
     <t>['transit_station', 'point_of_interest', 'establishment']</t>
   </si>
   <si>
@@ -613,15 +604,6 @@
     <t>座間</t>
   </si>
   <si>
-    <t>Zama, Kanagawa, Japan</t>
-  </si>
-  <si>
-    <t>{'location': {'lat': 35.480919, 'lng': 139.399888}, 'viewport': {'northeast': {'lat': 35.48226702989272, 'lng': 139.4011677298927}, 'southwest': {'lat': 35.47956737010728, 'lng': 139.3984680701073}}}</t>
-  </si>
-  <si>
-    <t>ChIJ14_WIJn_GGARRBsULuIuKlQ</t>
-  </si>
-  <si>
     <t>570 Kamigo, Ebina, Kanagawa 243-0434, Japan</t>
   </si>
   <si>
@@ -838,18 +820,9 @@
     <t>螢田</t>
   </si>
   <si>
-    <t>Takenoshita, Oyama, Sunto District, Shizuoka 410-1313, Japan</t>
-  </si>
-  <si>
-    <t>{'location': {'lat': 35.3332184, 'lng': 138.9812579}, 'viewport': {'northeast': {'lat': 35.33446047989273, 'lng': 138.9826119298927}, 'southwest': {'lat': 35.33176082010728, 'lng': 138.9799122701072}}}</t>
-  </si>
-  <si>
     <t>Ashigara Station</t>
   </si>
   <si>
-    <t>ChIJrcHuh0p0GWARAYU1-oqloOs</t>
-  </si>
-  <si>
     <t>OH46</t>
   </si>
   <si>
@@ -1234,9 +1207,6 @@
     <t>栗平</t>
   </si>
   <si>
-    <t>3 Chome Shiromidori, Kita Ward, Nagoya, Aichi 462-0046, Japan</t>
-  </si>
-  <si>
     <t>{'location': {'lat': 35.1971928, 'lng': 136.9101131}, 'viewport': {'northeast': {'lat': 35.19875527989272, 'lng': 136.91234105}, 'southwest': {'lat': 35.19605562010728, 'lng': 136.90826485}}}</t>
   </si>
   <si>
@@ -1255,15 +1225,6 @@
     <t>黒川</t>
   </si>
   <si>
-    <t>Kita Ward, Nagoya, Aichi, Japan</t>
-  </si>
-  <si>
-    <t>{'location': {'lat': 35.197193, 'lng': 136.910113}, 'viewport': {'northeast': {'lat': 35.19856022989272, 'lng': 136.9114629298928}, 'southwest': {'lat': 35.19586057010728, 'lng': 136.9087632701073}}}</t>
-  </si>
-  <si>
-    <t>ChIJg_v3J0lxA2AR99XaW6Vx7sE</t>
-  </si>
-  <si>
     <t>5 Chome-8-1 Haruhino, Asao-ku, Kawasaki, Kanagawa 215-0036, Japan</t>
   </si>
   <si>
@@ -1442,6 +1403,10 @@
   </si>
   <si>
     <t>小田急多摩センター</t>
+  </si>
+  <si>
+    <t>4 Minamikurokawa, Asao-ku, Kawasaki, Kanagawa 215-0034日本</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1813,10 +1778,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="3" max="3" width="29" customWidth="1"/>
+    <col min="9" max="9" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1885,31 +1851,31 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F3">
-        <v>35.690553899999998</v>
+        <v>35.683689399999999</v>
       </c>
       <c r="G3">
-        <v>139.69954989999999</v>
+        <v>139.6989165</v>
       </c>
       <c r="H3" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I3" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="J3" t="s">
         <v>17</v>
@@ -1917,31 +1883,31 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F4">
-        <v>35.683689399999999</v>
+        <v>35.678657700000002</v>
       </c>
       <c r="G4">
-        <v>139.6989165</v>
+        <v>139.6935182</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="J4" t="s">
         <v>17</v>
@@ -1949,31 +1915,31 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F5">
-        <v>35.678657700000002</v>
+        <v>35.669550200000003</v>
       </c>
       <c r="G5">
-        <v>139.6935182</v>
+        <v>139.6886476</v>
       </c>
       <c r="H5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="J5" t="s">
         <v>17</v>
@@ -1981,31 +1947,31 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="F6">
-        <v>35.669550200000003</v>
+        <v>35.669002599999999</v>
       </c>
       <c r="G6">
-        <v>139.6886476</v>
+        <v>139.67973319999999</v>
       </c>
       <c r="H6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J6" t="s">
         <v>17</v>
@@ -2013,31 +1979,31 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="F7">
-        <v>35.669002599999999</v>
+        <v>35.6654689</v>
       </c>
       <c r="G7">
-        <v>139.67973319999999</v>
+        <v>139.67305899999999</v>
       </c>
       <c r="H7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="I7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J7" t="s">
         <v>17</v>
@@ -2045,31 +2011,31 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F8">
-        <v>35.6654689</v>
+        <v>35.6615848</v>
       </c>
       <c r="G8">
-        <v>139.67305899999999</v>
+        <v>139.6668918</v>
       </c>
       <c r="H8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I8" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="J8" t="s">
         <v>17</v>
@@ -2077,31 +2043,31 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F9">
-        <v>35.6615848</v>
+        <v>35.6582291</v>
       </c>
       <c r="G9">
-        <v>139.6668918</v>
+        <v>139.66130229999999</v>
       </c>
       <c r="H9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J9" t="s">
         <v>17</v>
@@ -2109,31 +2075,31 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F10">
-        <v>35.6582291</v>
+        <v>35.655919799999999</v>
       </c>
       <c r="G10">
-        <v>139.66130229999999</v>
+        <v>139.65358359999999</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I10" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="J10" t="s">
         <v>17</v>
@@ -2141,31 +2107,31 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F11">
-        <v>35.655919799999999</v>
+        <v>35.653651799999999</v>
       </c>
       <c r="G11">
-        <v>139.65358359999999</v>
+        <v>139.64742219999999</v>
       </c>
       <c r="H11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="J11" t="s">
         <v>17</v>
@@ -2173,31 +2139,31 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C12" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F12">
-        <v>35.653651799999999</v>
+        <v>35.651207999999997</v>
       </c>
       <c r="G12">
-        <v>139.64742219999999</v>
+        <v>139.63680590000001</v>
       </c>
       <c r="H12" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I12" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="J12" t="s">
         <v>17</v>
@@ -2205,31 +2171,31 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C13" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D13" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F13">
-        <v>35.651207999999997</v>
+        <v>35.647502000000003</v>
       </c>
       <c r="G13">
-        <v>139.63680590000001</v>
+        <v>139.62388429999999</v>
       </c>
       <c r="H13" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I13" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="J13" t="s">
         <v>17</v>
@@ -2237,31 +2203,31 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C14" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D14" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E14" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F14">
-        <v>35.647502000000003</v>
+        <v>35.643316400000003</v>
       </c>
       <c r="G14">
-        <v>139.62388429999999</v>
+        <v>139.6095789</v>
       </c>
       <c r="H14" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="I14" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="J14" t="s">
         <v>17</v>
@@ -2269,31 +2235,31 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D15" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E15" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F15">
-        <v>35.643316400000003</v>
+        <v>35.640128300000001</v>
       </c>
       <c r="G15">
-        <v>139.6095789</v>
+        <v>139.59908730000001</v>
       </c>
       <c r="H15" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="I15" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J15" t="s">
         <v>17</v>
@@ -2301,25 +2267,25 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D16" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="E16" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F16">
-        <v>35.640128300000001</v>
+        <v>35.636546699999997</v>
       </c>
       <c r="G16">
-        <v>139.59908730000001</v>
+        <v>139.58724480000001</v>
       </c>
       <c r="H16" t="s">
         <v>100</v>
@@ -2339,25 +2305,25 @@
         <v>106</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E17" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F17">
-        <v>35.636546699999997</v>
+        <v>35.632389600000003</v>
       </c>
       <c r="G17">
-        <v>139.58724480000001</v>
+        <v>139.57763800000001</v>
       </c>
       <c r="H17" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="I17" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="J17" t="s">
         <v>17</v>
@@ -2365,31 +2331,31 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D18" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E18" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F18">
-        <v>35.632389600000003</v>
+        <v>35.627284400000001</v>
       </c>
       <c r="G18">
-        <v>139.57763800000001</v>
+        <v>139.5737096</v>
       </c>
       <c r="H18" t="s">
-        <v>112</v>
+        <v>429</v>
       </c>
       <c r="I18" t="s">
-        <v>113</v>
+        <v>430</v>
       </c>
       <c r="J18" t="s">
         <v>17</v>
@@ -2397,31 +2363,31 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F19">
-        <v>35.627284400000001</v>
+        <v>35.620766199999998</v>
       </c>
       <c r="G19">
-        <v>139.5737096</v>
+        <v>139.5700976</v>
       </c>
       <c r="H19" t="s">
-        <v>442</v>
+        <v>119</v>
       </c>
       <c r="I19" t="s">
-        <v>443</v>
+        <v>120</v>
       </c>
       <c r="J19" t="s">
         <v>17</v>
@@ -2429,31 +2395,31 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B20" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C20" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D20" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E20" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F20">
-        <v>35.620766199999998</v>
+        <v>35.617169400000002</v>
       </c>
       <c r="G20">
-        <v>139.5700976</v>
+        <v>139.56456750000001</v>
       </c>
       <c r="H20" t="s">
-        <v>122</v>
+        <v>431</v>
       </c>
       <c r="I20" t="s">
-        <v>123</v>
+        <v>432</v>
       </c>
       <c r="J20" t="s">
         <v>17</v>
@@ -2461,31 +2427,31 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C21" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D21" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E21" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F21">
-        <v>35.617169400000002</v>
+        <v>35.615013599999997</v>
       </c>
       <c r="G21">
-        <v>139.56456750000001</v>
+        <v>139.5422351</v>
       </c>
       <c r="H21" t="s">
-        <v>444</v>
+        <v>129</v>
       </c>
       <c r="I21" t="s">
-        <v>445</v>
+        <v>130</v>
       </c>
       <c r="J21" t="s">
         <v>17</v>
@@ -2493,31 +2459,31 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B22" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C22" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D22" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E22" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F22">
-        <v>35.615013599999997</v>
+        <v>35.614766799999998</v>
       </c>
       <c r="G22">
-        <v>139.5422351</v>
+        <v>139.52793790000001</v>
       </c>
       <c r="H22" t="s">
-        <v>132</v>
+        <v>433</v>
       </c>
       <c r="I22" t="s">
-        <v>133</v>
+        <v>434</v>
       </c>
       <c r="J22" t="s">
         <v>17</v>
@@ -2525,31 +2491,31 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C23" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D23" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E23" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F23">
-        <v>35.614766799999998</v>
+        <v>35.609032999999997</v>
       </c>
       <c r="G23">
-        <v>139.52793790000001</v>
+        <v>139.51616250000001</v>
       </c>
       <c r="H23" t="s">
-        <v>446</v>
+        <v>139</v>
       </c>
       <c r="I23" t="s">
-        <v>447</v>
+        <v>140</v>
       </c>
       <c r="J23" t="s">
         <v>17</v>
@@ -2557,31 +2523,31 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B24" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C24" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D24" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E24" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F24">
-        <v>35.609032999999997</v>
+        <v>35.603805000000001</v>
       </c>
       <c r="G24">
-        <v>139.51616250000001</v>
+        <v>139.50760500000001</v>
       </c>
       <c r="H24" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I24" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J24" t="s">
         <v>17</v>
@@ -2589,31 +2555,31 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B25" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C25" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D25" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E25" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F25">
-        <v>35.603805000000001</v>
+        <v>35.589807299999997</v>
       </c>
       <c r="G25">
-        <v>139.50760500000001</v>
+        <v>139.49793070000001</v>
       </c>
       <c r="H25" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I25" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J25" t="s">
         <v>17</v>
@@ -2621,31 +2587,31 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B26" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C26" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D26" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E26" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F26">
-        <v>35.589807299999997</v>
+        <v>35.583125699999997</v>
       </c>
       <c r="G26">
-        <v>139.49793070000001</v>
+        <v>139.4813915</v>
       </c>
       <c r="H26" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="I26" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="J26" t="s">
         <v>17</v>
@@ -2653,31 +2619,31 @@
     </row>
     <row r="27" spans="1:10">
       <c r="A27" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B27" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C27" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D27" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E27" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F27">
-        <v>35.583125699999997</v>
+        <v>35.563345900000002</v>
       </c>
       <c r="G27">
-        <v>139.4813915</v>
+        <v>139.46332960000001</v>
       </c>
       <c r="H27" t="s">
-        <v>160</v>
+        <v>435</v>
       </c>
       <c r="I27" t="s">
-        <v>161</v>
+        <v>436</v>
       </c>
       <c r="J27" t="s">
         <v>17</v>
@@ -2685,31 +2651,31 @@
     </row>
     <row r="28" spans="1:10">
       <c r="A28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B28" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E28" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F28">
-        <v>35.563345900000002</v>
+        <v>35.541994099999997</v>
       </c>
       <c r="G28">
-        <v>139.46332960000001</v>
+        <v>139.4453761</v>
       </c>
       <c r="H28" t="s">
-        <v>448</v>
+        <v>167</v>
       </c>
       <c r="I28" t="s">
-        <v>449</v>
+        <v>168</v>
       </c>
       <c r="J28" t="s">
         <v>17</v>
@@ -2717,482 +2683,482 @@
     </row>
     <row r="29" spans="1:10">
       <c r="A29" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B29" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C29" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D29" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E29" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F29">
-        <v>35.541994099999997</v>
+        <v>35.532456600000003</v>
       </c>
       <c r="G29">
-        <v>139.4453761</v>
+        <v>139.43817010000001</v>
       </c>
       <c r="H29" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="I29" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="J29" t="s">
-        <v>17</v>
+        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B30" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C30" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D30" t="s">
+        <v>179</v>
+      </c>
+      <c r="E30" t="s">
+        <v>23</v>
+      </c>
+      <c r="F30">
+        <v>35.515191199999997</v>
+      </c>
+      <c r="G30">
+        <v>139.4226534</v>
+      </c>
+      <c r="H30" t="s">
+        <v>180</v>
+      </c>
+      <c r="I30" t="s">
+        <v>181</v>
+      </c>
+      <c r="J30" t="s">
         <v>175</v>
-      </c>
-      <c r="E30" t="s">
-        <v>26</v>
-      </c>
-      <c r="F30">
-        <v>35.532456600000003</v>
-      </c>
-      <c r="G30">
-        <v>139.43817010000001</v>
-      </c>
-      <c r="H30" t="s">
-        <v>176</v>
-      </c>
-      <c r="I30" t="s">
-        <v>177</v>
-      </c>
-      <c r="J30" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B31" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C31" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D31" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="E31" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F31">
-        <v>35.515191199999997</v>
+        <v>35.499149500000001</v>
       </c>
       <c r="G31">
-        <v>139.4226534</v>
+        <v>139.40840549999999</v>
       </c>
       <c r="H31" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="I31" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="J31" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B32" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C32" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D32" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E32" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F32">
-        <v>35.499149500000001</v>
+        <v>35.480657000000001</v>
       </c>
       <c r="G32">
-        <v>139.40840549999999</v>
+        <v>139.39997260000001</v>
       </c>
       <c r="H32" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="I32" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="J32" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B33" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C33" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D33" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E33" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F33">
-        <v>35.480657000000001</v>
+        <v>35.452569099999998</v>
       </c>
       <c r="G33">
-        <v>139.39997260000001</v>
+        <v>139.39097520000001</v>
       </c>
       <c r="H33" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="I33" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="J33" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B34" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C34" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="D34" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="E34" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F34">
-        <v>35.480919</v>
+        <v>35.443379499999999</v>
       </c>
       <c r="G34">
-        <v>139.399888</v>
+        <v>139.37842739999999</v>
       </c>
       <c r="H34" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="I34" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="J34" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="B35" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="C35" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="D35" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="E35" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F35">
-        <v>35.452569099999998</v>
+        <v>35.439408299999997</v>
       </c>
       <c r="G35">
-        <v>139.39097520000001</v>
+        <v>139.36442210000001</v>
       </c>
       <c r="H35" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="I35" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="J35" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="B36" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C36" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D36" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="E36" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F36">
-        <v>35.443379499999999</v>
+        <v>35.417618599999997</v>
       </c>
       <c r="G36">
-        <v>139.37842739999999</v>
+        <v>139.3439673</v>
       </c>
       <c r="H36" t="s">
-        <v>210</v>
+        <v>437</v>
       </c>
       <c r="I36" t="s">
-        <v>211</v>
+        <v>438</v>
       </c>
       <c r="J36" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B37" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C37" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D37" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E37" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F37">
-        <v>35.439408299999997</v>
+        <v>35.396037100000001</v>
       </c>
       <c r="G37">
-        <v>139.36442210000001</v>
+        <v>139.3135935</v>
       </c>
       <c r="H37" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="I37" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="J37" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B38" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C38" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="D38" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="E38" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F38">
-        <v>35.417618599999997</v>
+        <v>35.381151699999997</v>
       </c>
       <c r="G38">
-        <v>139.3439673</v>
+        <v>139.27785589999999</v>
       </c>
       <c r="H38" t="s">
-        <v>450</v>
+        <v>439</v>
       </c>
       <c r="I38" t="s">
-        <v>451</v>
+        <v>440</v>
       </c>
       <c r="J38" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B39" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C39" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="D39" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="E39" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F39">
-        <v>35.396037100000001</v>
+        <v>35.373189500000002</v>
       </c>
       <c r="G39">
-        <v>139.3135935</v>
+        <v>139.27127960000001</v>
       </c>
       <c r="H39" t="s">
-        <v>226</v>
+        <v>441</v>
       </c>
       <c r="I39" t="s">
-        <v>227</v>
+        <v>442</v>
       </c>
       <c r="J39" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B40" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C40" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D40" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E40" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F40">
-        <v>35.381151699999997</v>
+        <v>35.370207600000001</v>
       </c>
       <c r="G40">
-        <v>139.27785589999999</v>
+        <v>139.22578290000001</v>
       </c>
       <c r="H40" t="s">
-        <v>452</v>
+        <v>234</v>
       </c>
       <c r="I40" t="s">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="J40" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B41" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C41" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D41" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E41" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F41">
-        <v>35.373189500000002</v>
+        <v>35.374168599999997</v>
       </c>
       <c r="G41">
-        <v>139.27127960000001</v>
+        <v>139.18456159999999</v>
       </c>
       <c r="H41" t="s">
-        <v>454</v>
+        <v>240</v>
       </c>
       <c r="I41" t="s">
-        <v>455</v>
+        <v>241</v>
       </c>
       <c r="J41" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B42" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="C42" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="D42" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="E42" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F42">
-        <v>35.370207600000001</v>
+        <v>35.344593799999998</v>
       </c>
       <c r="G42">
-        <v>139.22578290000001</v>
+        <v>139.13944359999999</v>
       </c>
       <c r="H42" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="I42" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="J42" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" t="s">
-        <v>242</v>
+        <v>423</v>
       </c>
       <c r="B43" t="s">
-        <v>243</v>
+        <v>424</v>
       </c>
       <c r="C43" t="s">
-        <v>244</v>
+        <v>425</v>
       </c>
       <c r="D43" t="s">
-        <v>245</v>
+        <v>426</v>
       </c>
       <c r="E43" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F43">
-        <v>35.374168599999997</v>
+        <v>35.326484999999998</v>
       </c>
       <c r="G43">
-        <v>139.18456159999999</v>
+        <v>139.135806</v>
       </c>
       <c r="H43" t="s">
-        <v>246</v>
+        <v>427</v>
       </c>
       <c r="I43" t="s">
-        <v>247</v>
+        <v>428</v>
       </c>
       <c r="J43" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -3209,13 +3175,13 @@
         <v>251</v>
       </c>
       <c r="E44" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F44">
-        <v>35.344593799999998</v>
+        <v>35.310425299999999</v>
       </c>
       <c r="G44">
-        <v>139.13944359999999</v>
+        <v>139.1427285</v>
       </c>
       <c r="H44" t="s">
         <v>252</v>
@@ -3224,1127 +3190,999 @@
         <v>253</v>
       </c>
       <c r="J44" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" t="s">
-        <v>436</v>
+        <v>254</v>
       </c>
       <c r="B45" t="s">
-        <v>437</v>
+        <v>255</v>
       </c>
       <c r="C45" t="s">
-        <v>438</v>
+        <v>256</v>
       </c>
       <c r="D45" t="s">
-        <v>439</v>
+        <v>257</v>
       </c>
       <c r="E45" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F45">
-        <v>35.326484999999998</v>
+        <v>35.296214399999997</v>
       </c>
       <c r="G45">
-        <v>139.135806</v>
+        <v>139.1455158</v>
       </c>
       <c r="H45" t="s">
-        <v>440</v>
+        <v>258</v>
       </c>
       <c r="I45" t="s">
-        <v>441</v>
+        <v>259</v>
       </c>
       <c r="J45" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="B46" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="C46" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="D46" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="E46" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F46">
-        <v>35.310425299999999</v>
+        <v>35.2850544</v>
       </c>
       <c r="G46">
-        <v>139.1427285</v>
+        <v>139.15199139999999</v>
       </c>
       <c r="H46" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="I46" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="J46" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="B47" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C47" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D47" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="E47" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F47">
-        <v>35.296214399999997</v>
+        <v>35.272165100000002</v>
       </c>
       <c r="G47">
-        <v>139.1455158</v>
+        <v>139.1545376</v>
       </c>
       <c r="H47" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="I47" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="J47" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B48" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="C48" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D48" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="E48" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F48">
-        <v>35.2850544</v>
+        <v>35.256444899999998</v>
       </c>
       <c r="G48">
-        <v>139.15199139999999</v>
+        <v>139.15539319999999</v>
       </c>
       <c r="H48" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="I48" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="J48" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="B49" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="C49" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="D49" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="E49" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F49">
-        <v>35.3332184</v>
+        <v>35.245435000000001</v>
       </c>
       <c r="G49">
-        <v>138.9812579</v>
+        <v>139.144811</v>
       </c>
       <c r="H49" t="s">
-        <v>276</v>
+        <v>443</v>
       </c>
       <c r="I49" t="s">
-        <v>277</v>
+        <v>444</v>
       </c>
       <c r="J49" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B50" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C50" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="D50" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="E50" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F50">
-        <v>35.272165100000002</v>
+        <v>35.246243499999999</v>
       </c>
       <c r="G50">
-        <v>139.1545376</v>
+        <v>139.12919830000001</v>
       </c>
       <c r="H50" t="s">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="I50" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="J50" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="B51" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="C51" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="D51" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="E51" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F51">
-        <v>35.256444899999998</v>
+        <v>35.240928099999998</v>
       </c>
       <c r="G51">
-        <v>139.15539319999999</v>
+        <v>139.12112999999999</v>
       </c>
       <c r="H51" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="I51" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="J51" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="B52" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="C52" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D52" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="E52" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F52">
-        <v>35.245435000000001</v>
+        <v>35.233281599999998</v>
       </c>
       <c r="G52">
-        <v>139.144811</v>
+        <v>139.10358780000001</v>
       </c>
       <c r="H52" t="s">
-        <v>456</v>
+        <v>298</v>
       </c>
       <c r="I52" t="s">
-        <v>457</v>
+        <v>299</v>
       </c>
       <c r="J52" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="B53" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="C53" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="D53" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="E53" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F53">
-        <v>35.246243499999999</v>
+        <v>35.520514899999988</v>
       </c>
       <c r="G53">
-        <v>139.12919830000001</v>
+        <v>139.4389007</v>
       </c>
       <c r="H53" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="I53" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="J53" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="B54" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="C54" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="D54" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="E54" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F54">
-        <v>35.240928099999998</v>
+        <v>35.508027900000002</v>
       </c>
       <c r="G54">
-        <v>139.12112999999999</v>
+        <v>139.44410579999999</v>
       </c>
       <c r="H54" t="s">
-        <v>301</v>
+        <v>445</v>
       </c>
       <c r="I54" t="s">
-        <v>302</v>
+        <v>446</v>
       </c>
       <c r="J54" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="B55" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="C55" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="D55" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="E55" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F55">
-        <v>35.233281599999998</v>
+        <v>35.495729400000002</v>
       </c>
       <c r="G55">
-        <v>139.10358780000001</v>
+        <v>139.447992</v>
       </c>
       <c r="H55" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="I55" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="J55" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B56" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C56" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="D56" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="E56" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F56">
-        <v>35.520514899999988</v>
+        <v>35.490214799999997</v>
       </c>
       <c r="G56">
-        <v>139.4389007</v>
+        <v>139.45082260000001</v>
       </c>
       <c r="H56" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="I56" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="J56" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B57" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="C57" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="D57" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="E57" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F57">
-        <v>35.508027900000002</v>
+        <v>35.4698305</v>
       </c>
       <c r="G57">
-        <v>139.44410579999999</v>
+        <v>139.46146340000001</v>
       </c>
       <c r="H57" t="s">
-        <v>458</v>
+        <v>326</v>
       </c>
       <c r="I57" t="s">
-        <v>459</v>
+        <v>327</v>
       </c>
       <c r="J57" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="B58" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="C58" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="D58" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="E58" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F58">
-        <v>35.495729400000002</v>
+        <v>35.450574699999997</v>
       </c>
       <c r="G58">
-        <v>139.447992</v>
+        <v>139.4657593</v>
       </c>
       <c r="H58" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="I58" t="s">
-        <v>324</v>
+        <v>333</v>
       </c>
       <c r="J58" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="B59" t="s">
-        <v>326</v>
+        <v>335</v>
       </c>
       <c r="C59" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
       <c r="D59" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="E59" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F59">
-        <v>35.490214799999997</v>
+        <v>35.432178800000003</v>
       </c>
       <c r="G59">
-        <v>139.45082260000001</v>
+        <v>139.46470600000001</v>
       </c>
       <c r="H59" t="s">
-        <v>329</v>
+        <v>447</v>
       </c>
       <c r="I59" t="s">
-        <v>330</v>
+        <v>448</v>
       </c>
       <c r="J59" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="B60" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="C60" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D60" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="E60" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F60">
-        <v>35.4698305</v>
+        <v>35.412521499999997</v>
       </c>
       <c r="G60">
-        <v>139.46146340000001</v>
+        <v>139.46547229999999</v>
       </c>
       <c r="H60" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="I60" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="J60" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="B61" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="C61" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="D61" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="E61" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="F61">
-        <v>35.450574699999997</v>
+        <v>35.396312299999998</v>
       </c>
       <c r="G61">
-        <v>139.4657593</v>
+        <v>139.46649260000001</v>
       </c>
       <c r="H61" t="s">
-        <v>341</v>
+        <v>449</v>
       </c>
       <c r="I61" t="s">
-        <v>342</v>
+        <v>450</v>
       </c>
       <c r="J61" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="B62" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="C62" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D62" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="E62" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F62">
-        <v>35.432178800000003</v>
+        <v>35.383503999999988</v>
       </c>
       <c r="G62">
-        <v>139.46470600000001</v>
+        <v>139.47084319999999</v>
       </c>
       <c r="H62" t="s">
-        <v>460</v>
+        <v>451</v>
       </c>
       <c r="I62" t="s">
-        <v>461</v>
+        <v>452</v>
       </c>
       <c r="J62" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B63" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="C63" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="D63" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="E63" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F63">
-        <v>35.412521499999997</v>
+        <v>35.362775800000001</v>
       </c>
       <c r="G63">
-        <v>139.46547229999999</v>
+        <v>139.47324710000001</v>
       </c>
       <c r="H63" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="I63" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="J63" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B64" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="C64" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D64" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="E64" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="F64">
-        <v>35.396312299999998</v>
+        <v>35.347993299999999</v>
       </c>
       <c r="G64">
-        <v>139.46649260000001</v>
+        <v>139.4762733</v>
       </c>
       <c r="H64" t="s">
-        <v>462</v>
+        <v>453</v>
       </c>
       <c r="I64" t="s">
-        <v>463</v>
+        <v>454</v>
       </c>
       <c r="J64" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="B65" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="C65" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="D65" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="E65" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F65">
-        <v>35.383503999999988</v>
+        <v>35.338898399999998</v>
       </c>
       <c r="G65">
-        <v>139.47084319999999</v>
+        <v>139.4874695</v>
       </c>
       <c r="H65" t="s">
-        <v>464</v>
+        <v>366</v>
       </c>
       <c r="I65" t="s">
-        <v>465</v>
+        <v>367</v>
       </c>
       <c r="J65" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="B66" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="C66" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="D66" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="E66" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F66">
-        <v>35.362775800000001</v>
+        <v>35.330786799999998</v>
       </c>
       <c r="G66">
-        <v>139.47324710000001</v>
+        <v>139.4748692</v>
       </c>
       <c r="H66" t="s">
-        <v>365</v>
+        <v>455</v>
       </c>
       <c r="I66" t="s">
-        <v>366</v>
+        <v>456</v>
       </c>
       <c r="J66" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="B67" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="C67" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="D67" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="E67" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F67">
-        <v>35.347993299999999</v>
+        <v>35.320791399999997</v>
       </c>
       <c r="G67">
-        <v>139.4762733</v>
+        <v>139.47107120000001</v>
       </c>
       <c r="H67" t="s">
-        <v>466</v>
+        <v>457</v>
       </c>
       <c r="I67" t="s">
-        <v>467</v>
+        <v>458</v>
       </c>
       <c r="J67" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="B68" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="C68" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="D68" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="E68" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F68">
-        <v>35.338898399999998</v>
+        <v>35.308772099999999</v>
       </c>
       <c r="G68">
-        <v>139.4874695</v>
+        <v>139.48348669999999</v>
       </c>
       <c r="H68" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="I68" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="J68" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="B69" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="C69" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="D69" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="E69" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F69">
-        <v>35.330786799999998</v>
+        <v>35.600150499999998</v>
       </c>
       <c r="G69">
-        <v>139.4748692</v>
+        <v>139.4936716</v>
       </c>
       <c r="H69" t="s">
-        <v>468</v>
+        <v>386</v>
       </c>
       <c r="I69" t="s">
-        <v>469</v>
+        <v>387</v>
       </c>
       <c r="J69" t="s">
-        <v>178</v>
+        <v>388</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="B70" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="C70" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="D70" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="E70" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F70">
-        <v>35.320791399999997</v>
+        <v>35.606028899999998</v>
       </c>
       <c r="G70">
-        <v>139.47107120000001</v>
+        <v>139.48091579999999</v>
       </c>
       <c r="H70" t="s">
-        <v>470</v>
+        <v>393</v>
       </c>
       <c r="I70" t="s">
-        <v>471</v>
+        <v>394</v>
       </c>
       <c r="J70" t="s">
-        <v>178</v>
+        <v>388</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" t="s">
-        <v>385</v>
+        <v>461</v>
       </c>
       <c r="B71" t="s">
-        <v>386</v>
+        <v>395</v>
       </c>
       <c r="C71" t="s">
-        <v>387</v>
+        <v>396</v>
       </c>
       <c r="D71" t="s">
+        <v>397</v>
+      </c>
+      <c r="E71" t="s">
+        <v>398</v>
+      </c>
+      <c r="F71">
+        <v>35.613320749676497</v>
+      </c>
+      <c r="G71">
+        <v>139.470802996218</v>
+      </c>
+      <c r="H71" t="s">
+        <v>399</v>
+      </c>
+      <c r="I71" t="s">
+        <v>400</v>
+      </c>
+      <c r="J71" t="s">
         <v>388</v>
-      </c>
-      <c r="E71" t="s">
-        <v>26</v>
-      </c>
-      <c r="F71">
-        <v>35.308772099999999</v>
-      </c>
-      <c r="G71">
-        <v>139.48348669999999</v>
-      </c>
-      <c r="H71" t="s">
-        <v>389</v>
-      </c>
-      <c r="I71" t="s">
-        <v>390</v>
-      </c>
-      <c r="J71" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" t="s">
-        <v>391</v>
+        <v>401</v>
       </c>
       <c r="B72" t="s">
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="C72" t="s">
-        <v>393</v>
+        <v>403</v>
       </c>
       <c r="D72" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
       <c r="E72" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F72">
-        <v>35.600150499999998</v>
+        <v>35.6188249</v>
       </c>
       <c r="G72">
-        <v>139.4936716</v>
+        <v>139.46464270000001</v>
       </c>
       <c r="H72" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
       <c r="I72" t="s">
-        <v>396</v>
+        <v>406</v>
       </c>
       <c r="J72" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
     </row>
     <row r="73" spans="1:10">
       <c r="A73" t="s">
-        <v>398</v>
+        <v>407</v>
       </c>
       <c r="B73" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
       <c r="C73" t="s">
-        <v>400</v>
+        <v>409</v>
       </c>
       <c r="D73" t="s">
-        <v>401</v>
+        <v>410</v>
       </c>
       <c r="E73" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F73">
-        <v>35.606028899999998</v>
+        <v>35.629930999999999</v>
       </c>
       <c r="G73">
-        <v>139.48091579999999</v>
+        <v>139.44801720000001</v>
       </c>
       <c r="H73" t="s">
-        <v>402</v>
+        <v>411</v>
       </c>
       <c r="I73" t="s">
-        <v>403</v>
+        <v>412</v>
       </c>
       <c r="J73" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" t="s">
-        <v>404</v>
+        <v>413</v>
       </c>
       <c r="B74" t="s">
-        <v>405</v>
+        <v>414</v>
       </c>
       <c r="C74" t="s">
-        <v>406</v>
+        <v>415</v>
       </c>
       <c r="D74" t="s">
-        <v>407</v>
+        <v>416</v>
       </c>
       <c r="E74" t="s">
-        <v>408</v>
+        <v>23</v>
       </c>
       <c r="F74">
-        <v>35.197192800000003</v>
+        <v>35.625065999999997</v>
       </c>
       <c r="G74">
-        <v>136.91011309999999</v>
+        <v>139.42453119999999</v>
       </c>
       <c r="H74" t="s">
-        <v>409</v>
+        <v>459</v>
       </c>
       <c r="I74" t="s">
-        <v>410</v>
+        <v>460</v>
       </c>
       <c r="J74" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="B75" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="C75" t="s">
-        <v>406</v>
+        <v>419</v>
       </c>
       <c r="D75" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="E75" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F75">
-        <v>35.197192999999999</v>
+        <v>35.615820300000003</v>
       </c>
       <c r="G75">
-        <v>136.910113</v>
+        <v>139.41111939999999</v>
       </c>
       <c r="H75" t="s">
-        <v>409</v>
+        <v>421</v>
       </c>
       <c r="I75" t="s">
-        <v>410</v>
+        <v>422</v>
       </c>
       <c r="J75" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10">
-      <c r="A76" t="s">
-        <v>414</v>
-      </c>
-      <c r="B76" t="s">
-        <v>415</v>
-      </c>
-      <c r="C76" t="s">
-        <v>416</v>
-      </c>
-      <c r="D76" t="s">
-        <v>417</v>
-      </c>
-      <c r="E76" t="s">
-        <v>26</v>
-      </c>
-      <c r="F76">
-        <v>35.6188249</v>
-      </c>
-      <c r="G76">
-        <v>139.46464270000001</v>
-      </c>
-      <c r="H76" t="s">
-        <v>418</v>
-      </c>
-      <c r="I76" t="s">
-        <v>419</v>
-      </c>
-      <c r="J76" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10">
-      <c r="A77" t="s">
-        <v>420</v>
-      </c>
-      <c r="B77" t="s">
-        <v>421</v>
-      </c>
-      <c r="C77" t="s">
-        <v>422</v>
-      </c>
-      <c r="D77" t="s">
-        <v>423</v>
-      </c>
-      <c r="E77" t="s">
-        <v>26</v>
-      </c>
-      <c r="F77">
-        <v>35.629930999999999</v>
-      </c>
-      <c r="G77">
-        <v>139.44801720000001</v>
-      </c>
-      <c r="H77" t="s">
-        <v>424</v>
-      </c>
-      <c r="I77" t="s">
-        <v>425</v>
-      </c>
-      <c r="J77" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10">
-      <c r="A78" t="s">
-        <v>426</v>
-      </c>
-      <c r="B78" t="s">
-        <v>427</v>
-      </c>
-      <c r="C78" t="s">
-        <v>428</v>
-      </c>
-      <c r="D78" t="s">
-        <v>429</v>
-      </c>
-      <c r="E78" t="s">
-        <v>26</v>
-      </c>
-      <c r="F78">
-        <v>35.625065999999997</v>
-      </c>
-      <c r="G78">
-        <v>139.42453119999999</v>
-      </c>
-      <c r="H78" t="s">
-        <v>472</v>
-      </c>
-      <c r="I78" t="s">
-        <v>473</v>
-      </c>
-      <c r="J78" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10">
-      <c r="A79" t="s">
-        <v>430</v>
-      </c>
-      <c r="B79" t="s">
-        <v>431</v>
-      </c>
-      <c r="C79" t="s">
-        <v>432</v>
-      </c>
-      <c r="D79" t="s">
-        <v>433</v>
-      </c>
-      <c r="E79" t="s">
-        <v>26</v>
-      </c>
-      <c r="F79">
-        <v>35.615820300000003</v>
-      </c>
-      <c r="G79">
-        <v>139.41111939999999</v>
-      </c>
-      <c r="H79" t="s">
-        <v>434</v>
-      </c>
-      <c r="I79" t="s">
-        <v>435</v>
-      </c>
-      <c r="J79" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>

</xml_diff>